<commit_message>
Activacion de "Recepción en el Dia" en Remitos, Recepciones. Mejoras generales de la interface. Botón Excel, etc.
</commit_message>
<xml_diff>
--- a/DOCS/REMITO_Master.xlsx
+++ b/DOCS/REMITO_Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORKS\CAPELLO SOMBREROS\APPLICATION\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDBC4ED2-CE68-4FA0-B5AF-F194EDB63983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E29DCCD3-CB09-4BDF-A9E4-998BD7C88E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -112,10 +112,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="_ [$€-2]\ * #,##0.00_ ;_ [$€-2]\ * \-#,##0.00_ ;_ [$€-2]\ * &quot;-&quot;??_ "/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="_ [$€-2]\ * #,##0.00_ ;_ [$€-2]\ * \-#,##0.00_ ;_ [$€-2]\ * &quot;-&quot;??_ "/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -363,8 +363,8 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -494,13 +494,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -845,9 +845,9 @@
   <dimension ref="A1:AR858"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" style="16" customWidth="1"/>
-    <col min="3" max="4" width="9" customWidth="1"/>
+    <col min="3" max="4" width="11.109375" customWidth="1"/>
     <col min="5" max="5" width="4.33203125" style="16" customWidth="1"/>
     <col min="6" max="7" width="4.33203125" customWidth="1"/>
     <col min="8" max="8" width="14.44140625" customWidth="1"/>

</xml_diff>

<commit_message>
Mejoras en Consulta de Remitos
</commit_message>
<xml_diff>
--- a/DOCS/REMITO_Master.xlsx
+++ b/DOCS/REMITO_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORKS\CAPELLO SOMBREROS\APPLICATION\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E29DCCD3-CB09-4BDF-A9E4-998BD7C88E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD09C8FA-28F2-4A65-BA06-EC140446469D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -117,7 +117,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="_ [$€-2]\ * #,##0.00_ ;_ [$€-2]\ * \-#,##0.00_ ;_ [$€-2]\ * &quot;-&quot;??_ "/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -135,12 +135,6 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
@@ -168,6 +162,18 @@
       <name val="Copperplate Gothic Bold"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <name val="STXingkai"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -363,10 +369,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -392,7 +398,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -404,10 +410,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -423,11 +429,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -435,7 +441,7 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -456,7 +462,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -475,7 +481,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -483,27 +489,26 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -513,19 +518,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -535,6 +540,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -863,30 +872,30 @@
       <c r="G1" s="9"/>
       <c r="H1" s="10"/>
     </row>
-    <row r="2" spans="1:17" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="51" t="s">
+    <row r="2" spans="1:17" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A2" s="70" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="50"/>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="56">
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="55">
         <v>0.7</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="58"/>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
+      <c r="A3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -900,28 +909,28 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="65"/>
-      <c r="B5" s="66"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="62" t="s">
+      <c r="A5" s="64"/>
+      <c r="B5" s="65"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="59"/>
+      <c r="G5" s="58"/>
       <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="67"/>
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="64"/>
+      <c r="A6" s="66"/>
+      <c r="B6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="63"/>
       <c r="F6" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="63"/>
-      <c r="H6" s="64"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="63"/>
     </row>
     <row r="7" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="24"/>
@@ -934,16 +943,16 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="68" t="s">
+      <c r="A8" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="69"/>
-      <c r="C8" s="69"/>
-      <c r="D8" s="69"/>
-      <c r="E8" s="69"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="57" t="s">
+      <c r="B8" s="68"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="56" t="s">
         <v>22</v>
       </c>
     </row>
@@ -978,11 +987,11 @@
     <row r="10" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="32"/>
       <c r="B10" s="25"/>
-      <c r="C10" s="54" t="str">
+      <c r="C10" s="53" t="str">
         <f>IF(D10 ="","",D10*$H$2)</f>
         <v/>
       </c>
-      <c r="D10" s="54"/>
+      <c r="D10" s="53"/>
       <c r="E10" s="32"/>
       <c r="F10" s="39"/>
       <c r="G10" s="39"/>
@@ -991,11 +1000,11 @@
     <row r="11" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="33"/>
       <c r="B11" s="25"/>
-      <c r="C11" s="54" t="str">
+      <c r="C11" s="53" t="str">
         <f t="shared" ref="C11:C34" si="0">IF(D11 ="","",D11*$H$2)</f>
         <v/>
       </c>
-      <c r="D11" s="54"/>
+      <c r="D11" s="53"/>
       <c r="E11" s="33"/>
       <c r="F11" s="40"/>
       <c r="G11" s="40"/>
@@ -1004,11 +1013,11 @@
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="34"/>
       <c r="B12" s="25"/>
-      <c r="C12" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D12" s="54"/>
+      <c r="C12" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D12" s="53"/>
       <c r="E12" s="41"/>
       <c r="F12" s="42"/>
       <c r="G12" s="43"/>
@@ -1017,11 +1026,11 @@
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="32"/>
       <c r="B13" s="25"/>
-      <c r="C13" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D13" s="54"/>
+      <c r="C13" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D13" s="53"/>
       <c r="E13" s="32"/>
       <c r="F13" s="37"/>
       <c r="G13" s="37"/>
@@ -1030,11 +1039,11 @@
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="32"/>
       <c r="B14" s="25"/>
-      <c r="C14" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D14" s="54"/>
+      <c r="C14" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D14" s="53"/>
       <c r="E14" s="32"/>
       <c r="F14" s="44"/>
       <c r="G14" s="44"/>
@@ -1043,11 +1052,11 @@
     <row r="15" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="32"/>
       <c r="B15" s="25"/>
-      <c r="C15" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D15" s="54"/>
+      <c r="C15" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D15" s="53"/>
       <c r="E15" s="32"/>
       <c r="F15" s="39"/>
       <c r="G15" s="39"/>
@@ -1056,11 +1065,11 @@
     <row r="16" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="32"/>
       <c r="B16" s="25"/>
-      <c r="C16" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D16" s="54"/>
+      <c r="C16" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D16" s="53"/>
       <c r="E16" s="32"/>
       <c r="F16" s="39"/>
       <c r="G16" s="39"/>
@@ -1069,11 +1078,11 @@
     <row r="17" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="32"/>
       <c r="B17" s="25"/>
-      <c r="C17" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D17" s="54"/>
+      <c r="C17" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D17" s="53"/>
       <c r="E17" s="32"/>
       <c r="F17" s="39"/>
       <c r="G17" s="39"/>
@@ -1082,11 +1091,11 @@
     <row r="18" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="32"/>
       <c r="B18" s="25"/>
-      <c r="C18" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D18" s="54"/>
+      <c r="C18" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D18" s="53"/>
       <c r="E18" s="32"/>
       <c r="F18" s="40"/>
       <c r="G18" s="40"/>
@@ -1095,11 +1104,11 @@
     <row r="19" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="35"/>
       <c r="B19" s="25"/>
-      <c r="C19" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D19" s="54"/>
+      <c r="C19" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D19" s="53"/>
       <c r="E19" s="33"/>
       <c r="F19" s="45"/>
       <c r="G19" s="45"/>
@@ -1108,11 +1117,11 @@
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="35"/>
       <c r="B20" s="25"/>
-      <c r="C20" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D20" s="54"/>
+      <c r="C20" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D20" s="53"/>
       <c r="E20" s="33"/>
       <c r="F20" s="37"/>
       <c r="G20" s="37"/>
@@ -1121,11 +1130,11 @@
     <row r="21" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="32"/>
       <c r="B21" s="25"/>
-      <c r="C21" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D21" s="54"/>
+      <c r="C21" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D21" s="53"/>
       <c r="E21" s="32"/>
       <c r="F21" s="39"/>
       <c r="G21" s="39"/>
@@ -1134,11 +1143,11 @@
     <row r="22" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="33"/>
       <c r="B22" s="25"/>
-      <c r="C22" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D22" s="54"/>
+      <c r="C22" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D22" s="53"/>
       <c r="E22" s="33"/>
       <c r="F22" s="40"/>
       <c r="G22" s="40"/>
@@ -1147,11 +1156,11 @@
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="36"/>
       <c r="B23" s="25"/>
-      <c r="C23" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D23" s="54"/>
+      <c r="C23" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D23" s="53"/>
       <c r="E23" s="33"/>
       <c r="F23" s="46"/>
       <c r="G23" s="46"/>
@@ -1160,11 +1169,11 @@
     <row r="24" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="32"/>
       <c r="B24" s="25"/>
-      <c r="C24" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D24" s="54"/>
+      <c r="C24" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D24" s="53"/>
       <c r="E24" s="32"/>
       <c r="F24" s="39"/>
       <c r="G24" s="39"/>
@@ -1173,11 +1182,11 @@
     <row r="25" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="32"/>
       <c r="B25" s="25"/>
-      <c r="C25" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D25" s="54"/>
+      <c r="C25" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D25" s="53"/>
       <c r="E25" s="33"/>
       <c r="F25" s="39"/>
       <c r="G25" s="39"/>
@@ -1186,11 +1195,11 @@
     <row r="26" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="33"/>
       <c r="B26" s="25"/>
-      <c r="C26" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D26" s="54"/>
+      <c r="C26" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D26" s="53"/>
       <c r="E26" s="47"/>
       <c r="F26" s="40"/>
       <c r="G26" s="40"/>
@@ -1199,11 +1208,11 @@
     <row r="27" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="32"/>
       <c r="B27" s="25"/>
-      <c r="C27" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D27" s="54"/>
+      <c r="C27" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D27" s="53"/>
       <c r="E27" s="32"/>
       <c r="F27" s="39"/>
       <c r="G27" s="39"/>
@@ -1212,11 +1221,11 @@
     <row r="28" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="32"/>
       <c r="B28" s="25"/>
-      <c r="C28" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D28" s="54"/>
+      <c r="C28" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D28" s="53"/>
       <c r="E28" s="32"/>
       <c r="F28" s="39"/>
       <c r="G28" s="39"/>
@@ -1225,11 +1234,11 @@
     <row r="29" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="32"/>
       <c r="B29" s="25"/>
-      <c r="C29" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D29" s="54"/>
+      <c r="C29" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D29" s="53"/>
       <c r="E29" s="32"/>
       <c r="F29" s="39"/>
       <c r="G29" s="39"/>
@@ -1238,11 +1247,11 @@
     <row r="30" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="32"/>
       <c r="B30" s="25"/>
-      <c r="C30" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D30" s="54"/>
+      <c r="C30" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D30" s="53"/>
       <c r="E30" s="32"/>
       <c r="F30" s="39"/>
       <c r="G30" s="39"/>
@@ -1251,11 +1260,11 @@
     <row r="31" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="32"/>
       <c r="B31" s="25"/>
-      <c r="C31" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D31" s="54"/>
+      <c r="C31" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D31" s="53"/>
       <c r="E31" s="32"/>
       <c r="F31" s="39"/>
       <c r="G31" s="39"/>
@@ -1264,11 +1273,11 @@
     <row r="32" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="32"/>
       <c r="B32" s="25"/>
-      <c r="C32" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D32" s="54"/>
+      <c r="C32" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D32" s="53"/>
       <c r="E32" s="32"/>
       <c r="F32" s="39"/>
       <c r="G32" s="39"/>
@@ -1277,11 +1286,11 @@
     <row r="33" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="32"/>
       <c r="B33" s="25"/>
-      <c r="C33" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D33" s="54"/>
+      <c r="C33" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D33" s="53"/>
       <c r="E33" s="32"/>
       <c r="F33" s="39"/>
       <c r="G33" s="39"/>
@@ -1290,11 +1299,11 @@
     <row r="34" spans="1:44" s="27" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="33"/>
       <c r="B34" s="17"/>
-      <c r="C34" s="55" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D34" s="55"/>
+      <c r="C34" s="54" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D34" s="54"/>
       <c r="E34" s="33"/>
       <c r="F34" s="40"/>
       <c r="G34" s="40"/>
@@ -1433,8 +1442,8 @@
       <c r="C43" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D43" s="60"/>
-      <c r="E43" s="61"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="60"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="5"/>

</xml_diff>

<commit_message>
mas mejoras y arreglo de bugs
</commit_message>
<xml_diff>
--- a/DOCS/REMITO_Master.xlsx
+++ b/DOCS/REMITO_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORKS\CAPELLO SOMBREROS\APPLICATION\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD09C8FA-28F2-4A65-BA06-EC140446469D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E80505-AF64-4493-A324-D5AFAD0B0F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Remito" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Remito!$A$1:$H$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Remito!$A$1:$H$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -98,13 +98,13 @@
     <t>Sombreros, Gorros y accesorios</t>
   </si>
   <si>
-    <t>CAPELLO</t>
-  </si>
-  <si>
     <t>REMITO DE MERCADERÍA EN CONSIGNACIÓN</t>
   </si>
   <si>
     <t>Nro.00000</t>
+  </si>
+  <si>
+    <t>Capello</t>
   </si>
 </sst>
 </file>
@@ -164,15 +164,15 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <sz val="36"/>
+      <name val="Edwardian Script ITC"/>
+      <family val="4"/>
     </font>
     <font>
       <b/>
-      <sz val="20"/>
-      <name val="STXingkai"/>
-      <charset val="134"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -189,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -338,17 +338,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -372,7 +361,7 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -402,7 +391,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -489,7 +477,7 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -540,10 +528,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -851,7 +839,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:AR858"/>
+  <dimension ref="A1:AR857"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.109375" customWidth="1"/>
@@ -872,34 +860,34 @@
       <c r="G1" s="9"/>
       <c r="H1" s="10"/>
     </row>
-    <row r="2" spans="1:17" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="70" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="50"/>
+    <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="1.05">
+      <c r="A2" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="49"/>
       <c r="C2" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="55">
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="54">
         <v>0.7</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="57"/>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
+      <c r="A3" s="56"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24"/>
+      <c r="A4" s="23"/>
       <c r="B4" s="15"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -909,31 +897,31 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="64"/>
-      <c r="B5" s="65"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="61" t="s">
+      <c r="A5" s="63"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="58"/>
-      <c r="H5" s="38"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="66"/>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="63"/>
+      <c r="A6" s="65"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="62"/>
       <c r="F6" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="62"/>
-      <c r="H6" s="63"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="62"/>
     </row>
     <row r="7" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="24"/>
+      <c r="A7" s="23"/>
       <c r="B7" s="15"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -943,21 +931,21 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="67" t="s">
+      <c r="A8" s="66" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="67"/>
+      <c r="C8" s="67"/>
+      <c r="D8" s="67"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="67"/>
+      <c r="H8" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="68"/>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="68"/>
-      <c r="H8" s="56" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="9" spans="1:17" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="29" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="13" t="s">
@@ -966,348 +954,348 @@
       <c r="C9" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="31" t="s">
+      <c r="D9" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="E9" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="30" t="s">
+      <c r="H9" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="22"/>
+      <c r="I9" s="21"/>
       <c r="Q9" s="2"/>
     </row>
     <row r="10" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="53" t="str">
+      <c r="A10" s="31"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="52" t="str">
         <f>IF(D10 ="","",D10*$H$2)</f>
         <v/>
       </c>
-      <c r="D10" s="53"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
+      <c r="D10" s="52"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
     </row>
     <row r="11" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="33"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="53" t="str">
+      <c r="A11" s="32"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="52" t="str">
         <f t="shared" ref="C11:C34" si="0">IF(D11 ="","",D11*$H$2)</f>
         <v/>
       </c>
-      <c r="D11" s="53"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="39"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D12" s="53"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="42"/>
+      <c r="A12" s="33"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D12" s="52"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="41"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D13" s="53"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="46"/>
+      <c r="A13" s="31"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D13" s="52"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="45"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D14" s="53"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="46"/>
+      <c r="A14" s="31"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D14" s="52"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="45"/>
     </row>
     <row r="15" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D15" s="53"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="40"/>
+      <c r="A15" s="31"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D15" s="52"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="39"/>
     </row>
     <row r="16" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="32"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D16" s="53"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="46"/>
+      <c r="A16" s="31"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D16" s="52"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="45"/>
     </row>
     <row r="17" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="32"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D17" s="53"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="49"/>
+      <c r="A17" s="31"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D17" s="52"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="48"/>
     </row>
     <row r="18" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D18" s="53"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
+      <c r="A18" s="31"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D18" s="52"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
     </row>
     <row r="19" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="35"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D19" s="53"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="40"/>
+      <c r="A19" s="34"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D19" s="52"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="44"/>
+      <c r="H19" s="39"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="35"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D20" s="53"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="46"/>
+      <c r="A20" s="34"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D20" s="52"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="45"/>
     </row>
     <row r="21" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D21" s="53"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="39"/>
+      <c r="A21" s="31"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D21" s="52"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
     </row>
     <row r="22" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="33"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D22" s="53"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
+      <c r="A22" s="32"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D22" s="52"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="36"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D23" s="53"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="42"/>
+      <c r="A23" s="35"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D23" s="52"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="41"/>
     </row>
     <row r="24" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D24" s="53"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="39"/>
+      <c r="A24" s="31"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D24" s="52"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="38"/>
     </row>
     <row r="25" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D25" s="53"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="39"/>
+      <c r="A25" s="31"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D25" s="52"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
     </row>
     <row r="26" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="33"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D26" s="53"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="40"/>
+      <c r="A26" s="32"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D26" s="52"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="39"/>
     </row>
     <row r="27" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="32"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D27" s="53"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="39"/>
+      <c r="A27" s="31"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D27" s="52"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
     </row>
     <row r="28" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="32"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D28" s="53"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
+      <c r="A28" s="31"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D28" s="52"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
     </row>
     <row r="29" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="32"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D29" s="53"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
+      <c r="A29" s="31"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D29" s="52"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
     </row>
     <row r="30" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D30" s="53"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="39"/>
-      <c r="H30" s="39"/>
+      <c r="A30" s="31"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D30" s="52"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
     </row>
     <row r="31" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D31" s="53"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="39"/>
-      <c r="G31" s="39"/>
-      <c r="H31" s="39"/>
+      <c r="A31" s="31"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D31" s="52"/>
+      <c r="E31" s="31"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
     </row>
     <row r="32" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D32" s="53"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="39"/>
-      <c r="H32" s="39"/>
+      <c r="A32" s="31"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D32" s="52"/>
+      <c r="E32" s="31"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
     </row>
     <row r="33" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D33" s="53"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-    </row>
-    <row r="34" spans="1:44" s="27" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="33"/>
+      <c r="A33" s="31"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="52" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D33" s="52"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+    </row>
+    <row r="34" spans="1:44" s="26" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="32"/>
       <c r="B34" s="17"/>
-      <c r="C34" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D34" s="54"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="40"/>
+      <c r="C34" s="53" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D34" s="53"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="39"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -1346,12 +1334,12 @@
       <c r="AR34"/>
     </row>
     <row r="35" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A35" s="20"/>
+      <c r="A35" s="19"/>
       <c r="C35" t="s">
         <v>15</v>
       </c>
       <c r="D35" s="5"/>
-      <c r="E35" s="41">
+      <c r="E35" s="40">
         <f>SUM(E10:E34)</f>
         <v>0</v>
       </c>
@@ -1364,11 +1352,11 @@
         <v>16</v>
       </c>
       <c r="D36" s="5"/>
-      <c r="E36" s="41">
+      <c r="E36" s="40">
         <f>SUM(F10:F34)</f>
         <v>0</v>
       </c>
-      <c r="H36" s="26"/>
+      <c r="H36" s="25"/>
     </row>
     <row r="37" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A37" s="11"/>
@@ -1377,13 +1365,13 @@
         <v>17</v>
       </c>
       <c r="D37" s="5"/>
-      <c r="E37" s="41">
+      <c r="E37" s="40">
         <f>SUM(G10:G34)</f>
         <v>0</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
-      <c r="H37" s="26"/>
+      <c r="H37" s="25"/>
     </row>
     <row r="38" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A38" s="11"/>
@@ -1399,7 +1387,7 @@
         <v>1</v>
       </c>
       <c r="D39" s="6"/>
-      <c r="E39" s="21"/>
+      <c r="E39" s="20"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
       <c r="H39" s="7"/>
@@ -1421,7 +1409,7 @@
         <v>2</v>
       </c>
       <c r="D41" s="6"/>
-      <c r="E41" s="21"/>
+      <c r="E41" s="20"/>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
       <c r="H41" s="7"/>
@@ -1442,14 +1430,14 @@
       <c r="C43" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D43" s="59"/>
-      <c r="E43" s="60"/>
+      <c r="D43" s="58"/>
+      <c r="E43" s="59"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="5"/>
     </row>
     <row r="44" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A44" s="23"/>
+      <c r="A44" s="22"/>
       <c r="B44" s="18"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
@@ -1465,9 +1453,9 @@
         <v>4</v>
       </c>
       <c r="D45" s="1"/>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="48"/>
+      <c r="E45" s="47"/>
+      <c r="F45" s="47"/>
+      <c r="G45" s="47"/>
       <c r="H45" s="5"/>
     </row>
     <row r="46" spans="1:44" x14ac:dyDescent="0.25">
@@ -1477,9 +1465,9 @@
         <v>5</v>
       </c>
       <c r="D46" s="1"/>
-      <c r="E46" s="36"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="48"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="47"/>
+      <c r="G46" s="47"/>
       <c r="H46" s="5"/>
     </row>
     <row r="47" spans="1:44" x14ac:dyDescent="0.25">
@@ -1502,18 +1490,8 @@
       <c r="G48" s="1"/>
       <c r="H48" s="5"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="19"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="21"/>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="7"/>
-    </row>
-    <row r="858" spans="10:10" x14ac:dyDescent="0.25">
-      <c r="J858" t="s">
+    <row r="857" spans="10:10" x14ac:dyDescent="0.25">
+      <c r="J857" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cambio de logo en el Remito
</commit_message>
<xml_diff>
--- a/DOCS/REMITO_Master.xlsx
+++ b/DOCS/REMITO_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORKS\CAPELLO SOMBREROS\APPLICATION\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E80505-AF64-4493-A324-D5AFAD0B0F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F4D1D0-9D95-499F-8D70-ECA5EC1B0B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -189,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -353,6 +353,17 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -480,27 +491,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -528,9 +526,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -861,30 +870,30 @@
       <c r="H1" s="10"/>
     </row>
     <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="1.05">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="69" t="s">
+      <c r="B2" s="66"/>
+      <c r="C2" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="54">
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="69">
         <v>0.7</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="56"/>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="4"/>
+      <c r="A3" s="63"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="64"/>
     </row>
     <row r="4" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="23"/>
@@ -897,28 +906,28 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="63"/>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="60" t="s">
+      <c r="A5" s="58"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="57"/>
+      <c r="G5" s="52"/>
       <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="65"/>
-      <c r="B6" s="64"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="64"/>
-      <c r="E6" s="62"/>
+      <c r="A6" s="60"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="57"/>
       <c r="F6" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="61"/>
-      <c r="H6" s="62"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="57"/>
     </row>
     <row r="7" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="23"/>
@@ -931,16 +940,16 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="66" t="s">
+      <c r="A8" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="67"/>
-      <c r="C8" s="67"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
-      <c r="G8" s="67"/>
-      <c r="H8" s="55" t="s">
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="51" t="s">
         <v>21</v>
       </c>
     </row>
@@ -975,11 +984,11 @@
     <row r="10" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="31"/>
       <c r="B10" s="24"/>
-      <c r="C10" s="52" t="str">
+      <c r="C10" s="49" t="str">
         <f>IF(D10 ="","",D10*$H$2)</f>
         <v/>
       </c>
-      <c r="D10" s="52"/>
+      <c r="D10" s="49"/>
       <c r="E10" s="31"/>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
@@ -988,11 +997,11 @@
     <row r="11" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="32"/>
       <c r="B11" s="24"/>
-      <c r="C11" s="52" t="str">
+      <c r="C11" s="49" t="str">
         <f t="shared" ref="C11:C34" si="0">IF(D11 ="","",D11*$H$2)</f>
         <v/>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="49"/>
       <c r="E11" s="32"/>
       <c r="F11" s="39"/>
       <c r="G11" s="39"/>
@@ -1001,11 +1010,11 @@
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="33"/>
       <c r="B12" s="24"/>
-      <c r="C12" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D12" s="52"/>
+      <c r="C12" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D12" s="49"/>
       <c r="E12" s="40"/>
       <c r="F12" s="41"/>
       <c r="G12" s="42"/>
@@ -1014,11 +1023,11 @@
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="31"/>
       <c r="B13" s="24"/>
-      <c r="C13" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D13" s="52"/>
+      <c r="C13" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D13" s="49"/>
       <c r="E13" s="31"/>
       <c r="F13" s="36"/>
       <c r="G13" s="36"/>
@@ -1027,11 +1036,11 @@
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="31"/>
       <c r="B14" s="24"/>
-      <c r="C14" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D14" s="52"/>
+      <c r="C14" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D14" s="49"/>
       <c r="E14" s="31"/>
       <c r="F14" s="43"/>
       <c r="G14" s="43"/>
@@ -1040,11 +1049,11 @@
     <row r="15" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="31"/>
       <c r="B15" s="24"/>
-      <c r="C15" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D15" s="52"/>
+      <c r="C15" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D15" s="49"/>
       <c r="E15" s="31"/>
       <c r="F15" s="38"/>
       <c r="G15" s="38"/>
@@ -1053,11 +1062,11 @@
     <row r="16" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="31"/>
       <c r="B16" s="24"/>
-      <c r="C16" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D16" s="52"/>
+      <c r="C16" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D16" s="49"/>
       <c r="E16" s="31"/>
       <c r="F16" s="38"/>
       <c r="G16" s="38"/>
@@ -1066,11 +1075,11 @@
     <row r="17" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="31"/>
       <c r="B17" s="24"/>
-      <c r="C17" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D17" s="52"/>
+      <c r="C17" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D17" s="49"/>
       <c r="E17" s="31"/>
       <c r="F17" s="38"/>
       <c r="G17" s="38"/>
@@ -1079,11 +1088,11 @@
     <row r="18" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31"/>
       <c r="B18" s="24"/>
-      <c r="C18" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D18" s="52"/>
+      <c r="C18" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D18" s="49"/>
       <c r="E18" s="31"/>
       <c r="F18" s="39"/>
       <c r="G18" s="39"/>
@@ -1092,11 +1101,11 @@
     <row r="19" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="34"/>
       <c r="B19" s="24"/>
-      <c r="C19" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D19" s="52"/>
+      <c r="C19" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D19" s="49"/>
       <c r="E19" s="32"/>
       <c r="F19" s="44"/>
       <c r="G19" s="44"/>
@@ -1105,11 +1114,11 @@
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="34"/>
       <c r="B20" s="24"/>
-      <c r="C20" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D20" s="52"/>
+      <c r="C20" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D20" s="49"/>
       <c r="E20" s="32"/>
       <c r="F20" s="36"/>
       <c r="G20" s="36"/>
@@ -1118,11 +1127,11 @@
     <row r="21" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="31"/>
       <c r="B21" s="24"/>
-      <c r="C21" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D21" s="52"/>
+      <c r="C21" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D21" s="49"/>
       <c r="E21" s="31"/>
       <c r="F21" s="38"/>
       <c r="G21" s="38"/>
@@ -1131,11 +1140,11 @@
     <row r="22" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32"/>
       <c r="B22" s="24"/>
-      <c r="C22" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D22" s="52"/>
+      <c r="C22" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D22" s="49"/>
       <c r="E22" s="32"/>
       <c r="F22" s="39"/>
       <c r="G22" s="39"/>
@@ -1144,11 +1153,11 @@
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="35"/>
       <c r="B23" s="24"/>
-      <c r="C23" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D23" s="52"/>
+      <c r="C23" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D23" s="49"/>
       <c r="E23" s="32"/>
       <c r="F23" s="45"/>
       <c r="G23" s="45"/>
@@ -1157,11 +1166,11 @@
     <row r="24" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="31"/>
       <c r="B24" s="24"/>
-      <c r="C24" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D24" s="52"/>
+      <c r="C24" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D24" s="49"/>
       <c r="E24" s="31"/>
       <c r="F24" s="38"/>
       <c r="G24" s="38"/>
@@ -1170,11 +1179,11 @@
     <row r="25" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="31"/>
       <c r="B25" s="24"/>
-      <c r="C25" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D25" s="52"/>
+      <c r="C25" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D25" s="49"/>
       <c r="E25" s="32"/>
       <c r="F25" s="38"/>
       <c r="G25" s="38"/>
@@ -1183,11 +1192,11 @@
     <row r="26" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="32"/>
       <c r="B26" s="24"/>
-      <c r="C26" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D26" s="52"/>
+      <c r="C26" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D26" s="49"/>
       <c r="E26" s="46"/>
       <c r="F26" s="39"/>
       <c r="G26" s="39"/>
@@ -1196,11 +1205,11 @@
     <row r="27" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="31"/>
       <c r="B27" s="24"/>
-      <c r="C27" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D27" s="52"/>
+      <c r="C27" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D27" s="49"/>
       <c r="E27" s="31"/>
       <c r="F27" s="38"/>
       <c r="G27" s="38"/>
@@ -1209,11 +1218,11 @@
     <row r="28" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="31"/>
       <c r="B28" s="24"/>
-      <c r="C28" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D28" s="52"/>
+      <c r="C28" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D28" s="49"/>
       <c r="E28" s="31"/>
       <c r="F28" s="38"/>
       <c r="G28" s="38"/>
@@ -1222,11 +1231,11 @@
     <row r="29" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="31"/>
       <c r="B29" s="24"/>
-      <c r="C29" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D29" s="52"/>
+      <c r="C29" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D29" s="49"/>
       <c r="E29" s="31"/>
       <c r="F29" s="38"/>
       <c r="G29" s="38"/>
@@ -1235,11 +1244,11 @@
     <row r="30" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="31"/>
       <c r="B30" s="24"/>
-      <c r="C30" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D30" s="52"/>
+      <c r="C30" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D30" s="49"/>
       <c r="E30" s="31"/>
       <c r="F30" s="38"/>
       <c r="G30" s="38"/>
@@ -1248,11 +1257,11 @@
     <row r="31" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="31"/>
       <c r="B31" s="24"/>
-      <c r="C31" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D31" s="52"/>
+      <c r="C31" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D31" s="49"/>
       <c r="E31" s="31"/>
       <c r="F31" s="38"/>
       <c r="G31" s="38"/>
@@ -1261,11 +1270,11 @@
     <row r="32" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="31"/>
       <c r="B32" s="24"/>
-      <c r="C32" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D32" s="52"/>
+      <c r="C32" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D32" s="49"/>
       <c r="E32" s="31"/>
       <c r="F32" s="38"/>
       <c r="G32" s="38"/>
@@ -1274,11 +1283,11 @@
     <row r="33" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="31"/>
       <c r="B33" s="24"/>
-      <c r="C33" s="52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D33" s="52"/>
+      <c r="C33" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D33" s="49"/>
       <c r="E33" s="31"/>
       <c r="F33" s="38"/>
       <c r="G33" s="38"/>
@@ -1287,11 +1296,11 @@
     <row r="34" spans="1:44" s="26" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="32"/>
       <c r="B34" s="17"/>
-      <c r="C34" s="53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D34" s="53"/>
+      <c r="C34" s="50" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D34" s="50"/>
       <c r="E34" s="32"/>
       <c r="F34" s="39"/>
       <c r="G34" s="39"/>
@@ -1430,8 +1439,8 @@
       <c r="C43" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D43" s="58"/>
-      <c r="E43" s="59"/>
+      <c r="D43" s="53"/>
+      <c r="E43" s="54"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="5"/>

</xml_diff>